<commit_message>
tender start data added
</commit_message>
<xml_diff>
--- a/tenders_start.xlsx
+++ b/tenders_start.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="274" documentId="8_{D8626B13-C0AC-4ED8-813A-C50E6300F95F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8325808F-5F64-4134-84AE-10AFB43E31BB}"/>
+  <xr:revisionPtr revIDLastSave="275" documentId="8_{D8626B13-C0AC-4ED8-813A-C50E6300F95F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C47F636-5DEC-49DC-9AF4-275FA99E0B66}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{2E88210F-F1DF-4337-AEAF-3D4D12C6EC05}"/>
   </bookViews>
@@ -160,15 +160,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -496,396 +495,395 @@
   <dimension ref="A1:N21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="32" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="1"/>
-    <col min="7" max="8" width="13.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" customWidth="1"/>
+    <col min="7" max="8" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="2">
+      <c r="D1" s="1">
         <v>1</v>
       </c>
-      <c r="E1" s="2">
+      <c r="E1" s="1">
         <v>2</v>
       </c>
-      <c r="F1" s="2">
+      <c r="F1" s="1">
         <v>3</v>
       </c>
-      <c r="G1" s="2">
+      <c r="G1" s="1">
         <v>4</v>
       </c>
-      <c r="H1" s="2">
+      <c r="H1" s="1">
         <v>5</v>
       </c>
-      <c r="I1" s="2">
+      <c r="I1" s="1">
         <v>6</v>
       </c>
-      <c r="J1" s="2">
+      <c r="J1" s="1">
         <v>7</v>
       </c>
-      <c r="K1" s="2">
+      <c r="K1" s="1">
         <v>8</v>
       </c>
-      <c r="L1" s="2">
+      <c r="L1" s="1">
         <v>9</v>
       </c>
-      <c r="M1" s="2">
+      <c r="M1" s="1">
         <v>10</v>
       </c>
-      <c r="N1" s="1">
+      <c r="N1">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2">
         <v>5</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2">
         <v>3625021.8558916501</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2">
         <v>3585241.2009922243</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2">
         <v>5242359.1716096196</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2">
         <v>0</v>
       </c>
-      <c r="H2" s="1">
+      <c r="H2">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3">
         <v>5</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3">
         <v>13464366.893311849</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3">
         <v>13316610.175113982</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3">
         <v>19471619.780264311</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G3">
         <v>51656909.241703324</v>
       </c>
-      <c r="H3" s="1">
+      <c r="H3">
         <v>65711883.688696265</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4">
         <v>5</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4">
         <v>0</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4">
         <v>0</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4">
         <v>0</v>
       </c>
-      <c r="G4" s="1">
+      <c r="G4">
         <v>13907629.411227813</v>
       </c>
-      <c r="H4" s="1">
+      <c r="H4">
         <v>17691660.993110523</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5">
         <v>2</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5">
         <v>43565104.360693097</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6">
         <v>2</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6">
         <v>40213942.486793622</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6">
         <v>111910967.15089689</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7">
         <v>1</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7">
         <v>13299464.00521188</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8">
         <v>3</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8">
         <v>13547121.107627736</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9">
         <v>3</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9">
         <v>12505034.868579449</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9">
         <v>26626398.679317039</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9">
         <v>25785425.000522137</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>2</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10">
         <v>1</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="3">
         <v>330279149.41895598</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>0</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11">
         <v>1</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11">
         <v>219201481.02228349</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12">
         <v>1</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12">
         <v>131520888.61337009</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13">
         <v>1</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13">
         <v>87680592.408913404</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14">
         <v>2</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14">
         <v>8948035.8691662811</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14">
         <v>9776403.551323479</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="A15" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>1</v>
       </c>
-      <c r="C15" s="1">
+      <c r="C15">
         <v>2</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15">
         <v>140931564.93936893</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15">
         <v>153978355.93334478</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="A16" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>9</v>
       </c>
-      <c r="C16" s="1">
+      <c r="C16">
         <v>2</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16">
         <v>17896071.738332562</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16">
         <v>19552807.102646958</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="A17" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="1">
+      <c r="C17">
         <v>2</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17">
         <v>31318125.542081982</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17">
         <v>34217412.429632172</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="A18" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>2</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18">
         <v>2</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18">
         <v>53688215.214997672</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18">
         <v>58658421.307940863</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="A19" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>0</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19">
         <v>1</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="3">
         <v>142479003.36778629</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="A20" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>5</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20">
         <v>1</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20">
         <v>180177056.35714662</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="A21" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>4</v>
       </c>
-      <c r="C21" s="1">
+      <c r="C21">
         <v>1</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21">
         <v>63305452.233592063</v>
       </c>
     </row>
@@ -898,6 +896,26 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="92d565b8-ba3a-4233-a05b-a1ab60ca7cf5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="fd2476d4-97b1-4075-989e-a063b18cae98" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010077DB98410970384A9A0497F576989D35" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="510ef340272b1c6d06523b37afa1120f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="92d565b8-ba3a-4233-a05b-a1ab60ca7cf5" xmlns:ns3="fd2476d4-97b1-4075-989e-a063b18cae98" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b1aa270078efd6d36fe11c333797bcf8" ns2:_="" ns3:_="">
     <xsd:import namespace="92d565b8-ba3a-4233-a05b-a1ab60ca7cf5"/>
@@ -1080,26 +1098,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="92d565b8-ba3a-4233-a05b-a1ab60ca7cf5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="fd2476d4-97b1-4075-989e-a063b18cae98" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B1FDD981-019F-40F5-9AB6-2DD33D8B65B2}">
   <ds:schemaRefs>
@@ -1109,6 +1107,25 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{926A699C-8A47-4BFC-B13A-1B438A677456}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="92d565b8-ba3a-4233-a05b-a1ab60ca7cf5"/>
+    <ds:schemaRef ds:uri="fd2476d4-97b1-4075-989e-a063b18cae98"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9106A6A0-1B4B-4B4E-B147-87C0CDE5B8BF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4663B556-36CB-41BA-9EF9-47ECC4BD6AF5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1127,25 +1144,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9106A6A0-1B4B-4B4E-B147-87C0CDE5B8BF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{926A699C-8A47-4BFC-B13A-1B438A677456}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="92d565b8-ba3a-4233-a05b-a1ab60ca7cf5"/>
-    <ds:schemaRef ds:uri="fd2476d4-97b1-4075-989e-a063b18cae98"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{79c742c4-e61c-4fa5-be89-a3cb566a80d1}" enabled="0" method="" siteId="{79c742c4-e61c-4fa5-be89-a3cb566a80d1}" removed="1"/>

</xml_diff>